<commit_message>
Petra hospital study v3: lean expandable Phase 1 as the base
Land leased, compact building with a structural provision for a third
floor, refurbished CT, leaner staffing and less debt. Full funding falls
from 7.48m to 5.82m JOD; adds option comparison and an upgrade path.
Version 2 kept under archive-v2-standard-build/.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaqwEyPcNCAyBboHzfJGfv
</commit_message>
<xml_diff>
--- a/feasibility-study-team-of-agents/studies/petra-trauma-hospital/model/PTC-financial-model.xlsx
+++ b/feasibility-study-team-of-agents/studies/petra-trauma-hospital/model/PTC-financial-model.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="26">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>160000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="31">
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>40000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="33">
@@ -761,250 +761,260 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>licence_fees</t>
+          <t>ground_rent</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>16000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>maint_building_pct</t>
+          <t>licence_fees</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>0.01</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cost_growth</t>
+          <t>maint_building_pct</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>0.025</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>maint_capex_pct</t>
+          <t>cost_growth</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>0.015</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>dso_days</t>
+          <t>maint_capex_pct</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>105</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>inventory_days</t>
+          <t>dso_days</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>payables_days</t>
+          <t>inventory_days</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>tax_rate</t>
+          <t>payables_days</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>0.21</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>tax_relief_pct</t>
+          <t>tax_rate</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>0.75</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>tax_relief_years</t>
+          <t>tax_relief_pct</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>discount_rate</t>
+          <t>tax_relief_years</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>0.1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>terminal_growth</t>
+          <t>discount_rate</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>0.02</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>t1_amount</t>
+          <t>terminal_growth</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>3000000</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>t1_rate</t>
+          <t>t1_amount</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>0.0375</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>t1_grace</t>
+          <t>t1_rate</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>2</v>
+        <v>0.0375</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>t1_repay</t>
+          <t>t1_grace</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>t2_amount</t>
+          <t>t1_repay</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>t2_rate</t>
+          <t>t2_amount</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>0.075</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>t2_grace</t>
+          <t>t2_rate</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>2</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>t2_repay</t>
+          <t>t2_grace</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>t3_amount</t>
+          <t>t2_repay</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>600000</v>
+        <v>8</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>t3_rate</t>
+          <t>t3_amount</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>t3_repay</t>
+          <t>t3_rate</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>5</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>cash_reserve</t>
+          <t>t3_repay</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>900000</v>
+        <v>5</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>cash_reserve</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>700000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>arrangement_fee_pct</t>
         </is>
       </c>
-      <c r="B58" s="2" t="n">
+      <c r="B59" s="2" t="n">
         <v>0.005</v>
       </c>
     </row>
@@ -1040,17 +1050,17 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>196200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Building (GFA x cost/m2)</t>
+          <t>Building (GFA x cost/m2, incl. expansion provision)</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1950000</v>
+        <v>1680000</v>
       </c>
     </row>
     <row r="5">
@@ -1060,7 +1070,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>117000</v>
+        <v>100800</v>
       </c>
     </row>
     <row r="6">
@@ -1070,7 +1080,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>380000</v>
+        <v>330000</v>
       </c>
     </row>
     <row r="7">
@@ -1080,7 +1090,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>1650000</v>
+        <v>1300000</v>
       </c>
     </row>
     <row r="8">
@@ -1090,7 +1100,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>200000</v>
+        <v>160000</v>
       </c>
     </row>
     <row r="9">
@@ -1100,7 +1110,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>90000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="10">
@@ -1110,7 +1120,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>398000</v>
+        <v>331000</v>
       </c>
     </row>
     <row r="11">
@@ -1120,7 +1130,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>320000</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="12">
@@ -1152,7 +1162,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>(Inputs!$B$46+Inputs!$B$50)*Inputs!$B$58</f>
+        <f>(Inputs!$B$47+Inputs!$B$51)*Inputs!$B$59</f>
         <v/>
       </c>
     </row>
@@ -1163,7 +1173,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>Inputs!$B$57</f>
+        <f>Inputs!$B$58</f>
         <v/>
       </c>
     </row>
@@ -1185,7 +1195,7 @@
         </is>
       </c>
       <c r="B17" s="3">
-        <f>Inputs!$B$46+Inputs!$B$50+Inputs!$B$54</f>
+        <f>Inputs!$B$47+Inputs!$B$51+Inputs!$B$55</f>
         <v/>
       </c>
     </row>
@@ -1230,7 +1240,7 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>2262000</v>
+        <v>1948800</v>
       </c>
       <c r="C22" t="n">
         <v>33</v>
@@ -1243,7 +1253,7 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>418000</v>
+        <v>363000</v>
       </c>
       <c r="C23" t="n">
         <v>10</v>
@@ -1256,7 +1266,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>1815000</v>
+        <v>1430000</v>
       </c>
       <c r="C24" t="n">
         <v>8</v>
@@ -1269,7 +1279,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>200000</v>
+        <v>160000</v>
       </c>
       <c r="C25" t="n">
         <v>5</v>
@@ -1282,7 +1292,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>90000</v>
+        <v>70000</v>
       </c>
       <c r="C26" t="n">
         <v>7</v>
@@ -1295,7 +1305,7 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>320000</v>
+        <v>280000</v>
       </c>
       <c r="C27" t="n">
         <v>5</v>
@@ -1739,10 +1749,10 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>0.95</v>
@@ -1887,7 +1897,7 @@
         </is>
       </c>
       <c r="B18" s="3">
-        <f>1229760*(1+Inputs!$B$23)</f>
+        <f>1096800*(1+Inputs!$B$23)</f>
         <v/>
       </c>
     </row>
@@ -2862,43 +2872,43 @@
         </is>
       </c>
       <c r="B22" s="3">
-        <f>Drivers!B$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!B$16</f>
+        <f>Drivers!B$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!B$16</f>
         <v/>
       </c>
       <c r="C22" s="3">
-        <f>Drivers!C$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!C$16</f>
+        <f>Drivers!C$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!C$16</f>
         <v/>
       </c>
       <c r="D22" s="3">
-        <f>Drivers!D$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!D$16</f>
+        <f>Drivers!D$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!D$16</f>
         <v/>
       </c>
       <c r="E22" s="3">
-        <f>Drivers!E$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!E$16</f>
+        <f>Drivers!E$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!E$16</f>
         <v/>
       </c>
       <c r="F22" s="3">
-        <f>Drivers!F$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!F$16</f>
+        <f>Drivers!F$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!F$16</f>
         <v/>
       </c>
       <c r="G22" s="3">
-        <f>Drivers!G$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!G$16</f>
+        <f>Drivers!G$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!G$16</f>
         <v/>
       </c>
       <c r="H22" s="3">
-        <f>Drivers!H$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!H$16</f>
+        <f>Drivers!H$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!H$16</f>
         <v/>
       </c>
       <c r="I22" s="3">
-        <f>Drivers!I$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!I$16</f>
+        <f>Drivers!I$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!I$16</f>
         <v/>
       </c>
       <c r="J22" s="3">
-        <f>Drivers!J$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!J$16</f>
+        <f>Drivers!J$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!J$16</f>
         <v/>
       </c>
       <c r="K22" s="3">
-        <f>Drivers!K$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$36)^Drivers!K$16</f>
+        <f>Drivers!K$9*Inputs!$B$21*Inputs!$B$28*(1+Inputs!$B$37)^Drivers!K$16</f>
         <v/>
       </c>
     </row>
@@ -2909,43 +2919,43 @@
         </is>
       </c>
       <c r="B23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!B$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!B$16</f>
         <v/>
       </c>
       <c r="C23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!C$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!C$16</f>
         <v/>
       </c>
       <c r="D23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!D$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!D$16</f>
         <v/>
       </c>
       <c r="E23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!E$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!E$16</f>
         <v/>
       </c>
       <c r="F23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!F$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!F$16</f>
         <v/>
       </c>
       <c r="G23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!G$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!G$16</f>
         <v/>
       </c>
       <c r="H23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!H$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!H$16</f>
         <v/>
       </c>
       <c r="I23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!I$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!I$16</f>
         <v/>
       </c>
       <c r="J23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!J$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!J$16</f>
         <v/>
       </c>
       <c r="K23" s="3">
-        <f>Inputs!$B$29*(1+Inputs!$B$36)^Drivers!K$16</f>
+        <f>Inputs!$B$29*(1+Inputs!$B$37)^Drivers!K$16</f>
         <v/>
       </c>
     </row>
@@ -2956,43 +2966,43 @@
         </is>
       </c>
       <c r="B24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!B$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!B$16</f>
         <v/>
       </c>
       <c r="C24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!C$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!C$16</f>
         <v/>
       </c>
       <c r="D24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!D$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!D$16</f>
         <v/>
       </c>
       <c r="E24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!E$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!E$16</f>
         <v/>
       </c>
       <c r="F24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!F$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!F$16</f>
         <v/>
       </c>
       <c r="G24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!G$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!G$16</f>
         <v/>
       </c>
       <c r="H24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!H$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!H$16</f>
         <v/>
       </c>
       <c r="I24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!I$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!I$16</f>
         <v/>
       </c>
       <c r="J24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!J$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!J$16</f>
         <v/>
       </c>
       <c r="K24" s="3">
-        <f>Inputs!$B$30*(1+Inputs!$B$36)^Drivers!K$16</f>
+        <f>Inputs!$B$30*(1+Inputs!$B$37)^Drivers!K$16</f>
         <v/>
       </c>
     </row>
@@ -3003,43 +3013,43 @@
         </is>
       </c>
       <c r="B25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!B$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!B$16</f>
         <v/>
       </c>
       <c r="C25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!C$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!C$16</f>
         <v/>
       </c>
       <c r="D25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!D$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!D$16</f>
         <v/>
       </c>
       <c r="E25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!E$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!E$16</f>
         <v/>
       </c>
       <c r="F25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!F$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!F$16</f>
         <v/>
       </c>
       <c r="G25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!G$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!G$16</f>
         <v/>
       </c>
       <c r="H25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!H$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!H$16</f>
         <v/>
       </c>
       <c r="I25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!I$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!I$16</f>
         <v/>
       </c>
       <c r="J25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!J$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!J$16</f>
         <v/>
       </c>
       <c r="K25" s="3">
-        <f>Inputs!$B$31*(1+Inputs!$B$36)^Drivers!K$16</f>
+        <f>Inputs!$B$31*(1+Inputs!$B$37)^Drivers!K$16</f>
         <v/>
       </c>
     </row>
@@ -3050,43 +3060,43 @@
         </is>
       </c>
       <c r="B26" s="3">
-        <f>Drivers!B$14*(1+Inputs!$B$36)^Drivers!B$16</f>
+        <f>Drivers!B$14*(1+Inputs!$B$37)^Drivers!B$16</f>
         <v/>
       </c>
       <c r="C26" s="3">
-        <f>Drivers!C$14*(1+Inputs!$B$36)^Drivers!C$16</f>
+        <f>Drivers!C$14*(1+Inputs!$B$37)^Drivers!C$16</f>
         <v/>
       </c>
       <c r="D26" s="3">
-        <f>Drivers!D$14*(1+Inputs!$B$36)^Drivers!D$16</f>
+        <f>Drivers!D$14*(1+Inputs!$B$37)^Drivers!D$16</f>
         <v/>
       </c>
       <c r="E26" s="3">
-        <f>Drivers!E$14*(1+Inputs!$B$36)^Drivers!E$16</f>
+        <f>Drivers!E$14*(1+Inputs!$B$37)^Drivers!E$16</f>
         <v/>
       </c>
       <c r="F26" s="3">
-        <f>Drivers!F$14*(1+Inputs!$B$36)^Drivers!F$16</f>
+        <f>Drivers!F$14*(1+Inputs!$B$37)^Drivers!F$16</f>
         <v/>
       </c>
       <c r="G26" s="3">
-        <f>Drivers!G$14*(1+Inputs!$B$36)^Drivers!G$16</f>
+        <f>Drivers!G$14*(1+Inputs!$B$37)^Drivers!G$16</f>
         <v/>
       </c>
       <c r="H26" s="3">
-        <f>Drivers!H$14*(1+Inputs!$B$36)^Drivers!H$16</f>
+        <f>Drivers!H$14*(1+Inputs!$B$37)^Drivers!H$16</f>
         <v/>
       </c>
       <c r="I26" s="3">
-        <f>Drivers!I$14*(1+Inputs!$B$36)^Drivers!I$16</f>
+        <f>Drivers!I$14*(1+Inputs!$B$37)^Drivers!I$16</f>
         <v/>
       </c>
       <c r="J26" s="3">
-        <f>Drivers!J$14*(1+Inputs!$B$36)^Drivers!J$16</f>
+        <f>Drivers!J$14*(1+Inputs!$B$37)^Drivers!J$16</f>
         <v/>
       </c>
       <c r="K26" s="3">
-        <f>Drivers!K$14*(1+Inputs!$B$36)^Drivers!K$16</f>
+        <f>Drivers!K$14*(1+Inputs!$B$37)^Drivers!K$16</f>
         <v/>
       </c>
     </row>
@@ -3097,43 +3107,43 @@
         </is>
       </c>
       <c r="B27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!B$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!B$16</f>
         <v/>
       </c>
       <c r="C27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!C$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!C$16</f>
         <v/>
       </c>
       <c r="D27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!D$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!D$16</f>
         <v/>
       </c>
       <c r="E27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!E$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!E$16</f>
         <v/>
       </c>
       <c r="F27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!F$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!F$16</f>
         <v/>
       </c>
       <c r="G27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!G$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!G$16</f>
         <v/>
       </c>
       <c r="H27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!H$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!H$16</f>
         <v/>
       </c>
       <c r="I27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!I$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!I$16</f>
         <v/>
       </c>
       <c r="J27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!J$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!J$16</f>
         <v/>
       </c>
       <c r="K27" s="3">
-        <f>Inputs!$B$32*(1+Inputs!$B$36)^Drivers!K$16</f>
+        <f>Inputs!$B$32*(1+Inputs!$B$37)^Drivers!K$16</f>
         <v/>
       </c>
     </row>
@@ -3144,43 +3154,43 @@
         </is>
       </c>
       <c r="B28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!B$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!B$16</f>
         <v/>
       </c>
       <c r="C28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!C$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!C$16</f>
         <v/>
       </c>
       <c r="D28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!D$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!D$16</f>
         <v/>
       </c>
       <c r="E28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!E$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!E$16</f>
         <v/>
       </c>
       <c r="F28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!F$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!F$16</f>
         <v/>
       </c>
       <c r="G28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!G$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!G$16</f>
         <v/>
       </c>
       <c r="H28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!H$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!H$16</f>
         <v/>
       </c>
       <c r="I28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!I$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!I$16</f>
         <v/>
       </c>
       <c r="J28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!J$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!J$16</f>
         <v/>
       </c>
       <c r="K28" s="3">
-        <f>Inputs!$B$33*(1+Inputs!$B$36)^Drivers!K$16</f>
+        <f>(Inputs!$B$33+Inputs!$B$34)*(1+Inputs!$B$37)^Drivers!K$16</f>
         <v/>
       </c>
     </row>
@@ -3191,43 +3201,43 @@
         </is>
       </c>
       <c r="B29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!B$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!B$16</f>
         <v/>
       </c>
       <c r="C29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!C$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!C$16</f>
         <v/>
       </c>
       <c r="D29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!D$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!D$16</f>
         <v/>
       </c>
       <c r="E29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!E$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!E$16</f>
         <v/>
       </c>
       <c r="F29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!F$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!F$16</f>
         <v/>
       </c>
       <c r="G29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!G$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!G$16</f>
         <v/>
       </c>
       <c r="H29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!H$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!H$16</f>
         <v/>
       </c>
       <c r="I29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!I$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!I$16</f>
         <v/>
       </c>
       <c r="J29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!J$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!J$16</f>
         <v/>
       </c>
       <c r="K29" s="3">
-        <f>Inputs!$B$34*(1+Inputs!$B$36)^Drivers!K$16</f>
+        <f>Inputs!$B$35*(1+Inputs!$B$37)^Drivers!K$16</f>
         <v/>
       </c>
     </row>
@@ -3238,43 +3248,43 @@
         </is>
       </c>
       <c r="B30" s="3">
-        <f>(Capex!$B$24*Drivers!B$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!B$16</f>
+        <f>(Capex!$B$24*Drivers!B$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!B$16</f>
         <v/>
       </c>
       <c r="C30" s="3">
-        <f>(Capex!$B$24*Drivers!C$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!C$16</f>
+        <f>(Capex!$B$24*Drivers!C$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!C$16</f>
         <v/>
       </c>
       <c r="D30" s="3">
-        <f>(Capex!$B$24*Drivers!D$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!D$16</f>
+        <f>(Capex!$B$24*Drivers!D$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!D$16</f>
         <v/>
       </c>
       <c r="E30" s="3">
-        <f>(Capex!$B$24*Drivers!E$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!E$16</f>
+        <f>(Capex!$B$24*Drivers!E$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!E$16</f>
         <v/>
       </c>
       <c r="F30" s="3">
-        <f>(Capex!$B$24*Drivers!F$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!F$16</f>
+        <f>(Capex!$B$24*Drivers!F$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!F$16</f>
         <v/>
       </c>
       <c r="G30" s="3">
-        <f>(Capex!$B$24*Drivers!G$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!G$16</f>
+        <f>(Capex!$B$24*Drivers!G$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!G$16</f>
         <v/>
       </c>
       <c r="H30" s="3">
-        <f>(Capex!$B$24*Drivers!H$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!H$16</f>
+        <f>(Capex!$B$24*Drivers!H$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!H$16</f>
         <v/>
       </c>
       <c r="I30" s="3">
-        <f>(Capex!$B$24*Drivers!I$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!I$16</f>
+        <f>(Capex!$B$24*Drivers!I$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!I$16</f>
         <v/>
       </c>
       <c r="J30" s="3">
-        <f>(Capex!$B$24*Drivers!J$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!J$16</f>
+        <f>(Capex!$B$24*Drivers!J$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!J$16</f>
         <v/>
       </c>
       <c r="K30" s="3">
-        <f>(Capex!$B$24*Drivers!K$15+Capex!$B$22*Inputs!$B$35)*(1+Inputs!$B$36)^Drivers!K$16</f>
+        <f>(Capex!$B$24*Drivers!K$15+Capex!$B$22*Inputs!$B$36)*(1+Inputs!$B$37)^Drivers!K$16</f>
         <v/>
       </c>
     </row>
@@ -3481,35 +3491,35 @@
         <v/>
       </c>
       <c r="D35" s="3">
-        <f>D17*Inputs!$B$37</f>
+        <f>D17*Inputs!$B$38</f>
         <v/>
       </c>
       <c r="E35" s="3">
-        <f>E17*Inputs!$B$37</f>
+        <f>E17*Inputs!$B$38</f>
         <v/>
       </c>
       <c r="F35" s="3">
-        <f>F17*Inputs!$B$37</f>
+        <f>F17*Inputs!$B$38</f>
         <v/>
       </c>
       <c r="G35" s="3">
-        <f>G17*Inputs!$B$37</f>
+        <f>G17*Inputs!$B$38</f>
         <v/>
       </c>
       <c r="H35" s="3">
-        <f>H17*Inputs!$B$37</f>
+        <f>H17*Inputs!$B$38</f>
         <v/>
       </c>
       <c r="I35" s="3">
-        <f>I17*Inputs!$B$37</f>
+        <f>I17*Inputs!$B$38</f>
         <v/>
       </c>
       <c r="J35" s="3">
-        <f>J17*Inputs!$B$37</f>
+        <f>J17*Inputs!$B$38</f>
         <v/>
       </c>
       <c r="K35" s="3">
-        <f>K17*Inputs!$B$37</f>
+        <f>K17*Inputs!$B$38</f>
         <v/>
       </c>
     </row>
@@ -3708,43 +3718,43 @@
         </is>
       </c>
       <c r="B40" s="3">
-        <f>MAX(B38+B39,0)*Inputs!$B$41*IF(Drivers!B$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(B38+B39,0)*Inputs!$B$42*IF(Drivers!B$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="C40" s="3">
-        <f>MAX(C38+C39,0)*Inputs!$B$41*IF(Drivers!C$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(C38+C39,0)*Inputs!$B$42*IF(Drivers!C$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="D40" s="3">
-        <f>MAX(D38+D39,0)*Inputs!$B$41*IF(Drivers!D$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(D38+D39,0)*Inputs!$B$42*IF(Drivers!D$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="E40" s="3">
-        <f>MAX(E38+E39,0)*Inputs!$B$41*IF(Drivers!E$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(E38+E39,0)*Inputs!$B$42*IF(Drivers!E$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="F40" s="3">
-        <f>MAX(F38+F39,0)*Inputs!$B$41*IF(Drivers!F$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(F38+F39,0)*Inputs!$B$42*IF(Drivers!F$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="G40" s="3">
-        <f>MAX(G38+G39,0)*Inputs!$B$41*IF(Drivers!G$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(G38+G39,0)*Inputs!$B$42*IF(Drivers!G$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="H40" s="3">
-        <f>MAX(H38+H39,0)*Inputs!$B$41*IF(Drivers!H$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(H38+H39,0)*Inputs!$B$42*IF(Drivers!H$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="I40" s="3">
-        <f>MAX(I38+I39,0)*Inputs!$B$41*IF(Drivers!I$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(I38+I39,0)*Inputs!$B$42*IF(Drivers!I$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="J40" s="3">
-        <f>MAX(J38+J39,0)*Inputs!$B$41*IF(Drivers!J$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(J38+J39,0)*Inputs!$B$42*IF(Drivers!J$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="K40" s="3">
-        <f>MAX(K38+K39,0)*Inputs!$B$41*IF(Drivers!K$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(K38+K39,0)*Inputs!$B$42*IF(Drivers!K$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
     </row>
@@ -3917,7 +3927,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>Inputs!$B$46</f>
+        <f>Inputs!$B$47</f>
         <v/>
       </c>
       <c r="C4" s="3">
@@ -3972,43 +3982,43 @@
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>IF(AND(1&gt;=Inputs!$B$48,1&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(1&gt;=Inputs!$B$49,1&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>IF(AND(2&gt;=Inputs!$B$48,2&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(2&gt;=Inputs!$B$49,2&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>IF(AND(3&gt;=Inputs!$B$48,3&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(3&gt;=Inputs!$B$49,3&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>IF(AND(4&gt;=Inputs!$B$48,4&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(4&gt;=Inputs!$B$49,4&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
       <c r="G5" s="3">
-        <f>IF(AND(5&gt;=Inputs!$B$48,5&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(5&gt;=Inputs!$B$49,5&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
       <c r="H5" s="3">
-        <f>IF(AND(6&gt;=Inputs!$B$48,6&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(6&gt;=Inputs!$B$49,6&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
       <c r="I5" s="3">
-        <f>IF(AND(7&gt;=Inputs!$B$48,7&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(7&gt;=Inputs!$B$49,7&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
       <c r="J5" s="3">
-        <f>IF(AND(8&gt;=Inputs!$B$48,8&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(8&gt;=Inputs!$B$49,8&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
       <c r="K5" s="3">
-        <f>IF(AND(9&gt;=Inputs!$B$48,9&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(9&gt;=Inputs!$B$49,9&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
       <c r="L5" s="3">
-        <f>IF(AND(10&gt;=Inputs!$B$48,10&lt;Inputs!$B$48+Inputs!$B$49),PMT(Inputs!$B$47,Inputs!$B$49,-Inputs!$B$46),0)</f>
+        <f>IF(AND(10&gt;=Inputs!$B$49,10&lt;Inputs!$B$49+Inputs!$B$50),PMT(Inputs!$B$48,Inputs!$B$50,-Inputs!$B$47),0)</f>
         <v/>
       </c>
     </row>
@@ -4019,47 +4029,47 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>B4*Inputs!$B$47*0.5</f>
+        <f>B4*Inputs!$B$48*0.5</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>C3*Inputs!$B$47</f>
+        <f>C3*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>D3*Inputs!$B$47</f>
+        <f>D3*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>E3*Inputs!$B$47</f>
+        <f>E3*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>F3*Inputs!$B$47</f>
+        <f>F3*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="G6" s="3">
-        <f>G3*Inputs!$B$47</f>
+        <f>G3*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="H6" s="3">
-        <f>H3*Inputs!$B$47</f>
+        <f>H3*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="I6" s="3">
-        <f>I3*Inputs!$B$47</f>
+        <f>I3*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="J6" s="3">
-        <f>J3*Inputs!$B$47</f>
+        <f>J3*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="K6" s="3">
-        <f>K3*Inputs!$B$47</f>
+        <f>K3*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="L6" s="3">
-        <f>L3*Inputs!$B$47</f>
+        <f>L3*Inputs!$B$48</f>
         <v/>
       </c>
     </row>
@@ -4263,7 +4273,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>Inputs!$B$50</f>
+        <f>Inputs!$B$51</f>
         <v/>
       </c>
       <c r="C12" s="3">
@@ -4318,43 +4328,43 @@
         <v/>
       </c>
       <c r="C13" s="3">
-        <f>IF(AND(1&gt;=Inputs!$B$52,1&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(1&gt;=Inputs!$B$53,1&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
       <c r="D13" s="3">
-        <f>IF(AND(2&gt;=Inputs!$B$52,2&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(2&gt;=Inputs!$B$53,2&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
       <c r="E13" s="3">
-        <f>IF(AND(3&gt;=Inputs!$B$52,3&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(3&gt;=Inputs!$B$53,3&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>IF(AND(4&gt;=Inputs!$B$52,4&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(4&gt;=Inputs!$B$53,4&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
       <c r="G13" s="3">
-        <f>IF(AND(5&gt;=Inputs!$B$52,5&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(5&gt;=Inputs!$B$53,5&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
       <c r="H13" s="3">
-        <f>IF(AND(6&gt;=Inputs!$B$52,6&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(6&gt;=Inputs!$B$53,6&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
       <c r="I13" s="3">
-        <f>IF(AND(7&gt;=Inputs!$B$52,7&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(7&gt;=Inputs!$B$53,7&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
       <c r="J13" s="3">
-        <f>IF(AND(8&gt;=Inputs!$B$52,8&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(8&gt;=Inputs!$B$53,8&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
       <c r="K13" s="3">
-        <f>IF(AND(9&gt;=Inputs!$B$52,9&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(9&gt;=Inputs!$B$53,9&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
       <c r="L13" s="3">
-        <f>IF(AND(10&gt;=Inputs!$B$52,10&lt;Inputs!$B$52+Inputs!$B$53),PMT(Inputs!$B$51,Inputs!$B$53,-Inputs!$B$50),0)</f>
+        <f>IF(AND(10&gt;=Inputs!$B$53,10&lt;Inputs!$B$53+Inputs!$B$54),PMT(Inputs!$B$52,Inputs!$B$54,-Inputs!$B$51),0)</f>
         <v/>
       </c>
     </row>
@@ -4365,47 +4375,47 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>B12*Inputs!$B$51*0.5</f>
+        <f>B12*Inputs!$B$52*0.5</f>
         <v/>
       </c>
       <c r="C14" s="3">
-        <f>C11*Inputs!$B$51</f>
+        <f>C11*Inputs!$B$52</f>
         <v/>
       </c>
       <c r="D14" s="3">
-        <f>D11*Inputs!$B$51</f>
+        <f>D11*Inputs!$B$52</f>
         <v/>
       </c>
       <c r="E14" s="3">
-        <f>E11*Inputs!$B$51</f>
+        <f>E11*Inputs!$B$52</f>
         <v/>
       </c>
       <c r="F14" s="3">
-        <f>F11*Inputs!$B$51</f>
+        <f>F11*Inputs!$B$52</f>
         <v/>
       </c>
       <c r="G14" s="3">
-        <f>G11*Inputs!$B$51</f>
+        <f>G11*Inputs!$B$52</f>
         <v/>
       </c>
       <c r="H14" s="3">
-        <f>H11*Inputs!$B$51</f>
+        <f>H11*Inputs!$B$52</f>
         <v/>
       </c>
       <c r="I14" s="3">
-        <f>I11*Inputs!$B$51</f>
+        <f>I11*Inputs!$B$52</f>
         <v/>
       </c>
       <c r="J14" s="3">
-        <f>J11*Inputs!$B$51</f>
+        <f>J11*Inputs!$B$52</f>
         <v/>
       </c>
       <c r="K14" s="3">
-        <f>K11*Inputs!$B$51</f>
+        <f>K11*Inputs!$B$52</f>
         <v/>
       </c>
       <c r="L14" s="3">
-        <f>L11*Inputs!$B$51</f>
+        <f>L11*Inputs!$B$52</f>
         <v/>
       </c>
     </row>
@@ -4609,7 +4619,7 @@
         </is>
       </c>
       <c r="B20" s="3">
-        <f>Inputs!$B$54</f>
+        <f>Inputs!$B$55</f>
         <v/>
       </c>
       <c r="C20" s="3">
@@ -4664,43 +4674,43 @@
         <v/>
       </c>
       <c r="C21" s="3">
-        <f>IF(1&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(1&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
       <c r="D21" s="3">
-        <f>IF(2&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(2&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
       <c r="E21" s="3">
-        <f>IF(3&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(3&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
       <c r="F21" s="3">
-        <f>IF(4&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(4&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
       <c r="G21" s="3">
-        <f>IF(5&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(5&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
       <c r="H21" s="3">
-        <f>IF(6&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(6&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
       <c r="I21" s="3">
-        <f>IF(7&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(7&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
       <c r="J21" s="3">
-        <f>IF(8&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(8&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
       <c r="K21" s="3">
-        <f>IF(9&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(9&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
       <c r="L21" s="3">
-        <f>IF(10&lt;=Inputs!$B$56,PMT(Inputs!$B$55,Inputs!$B$56,-Inputs!$B$54),0)</f>
+        <f>IF(10&lt;=Inputs!$B$57,PMT(Inputs!$B$56,Inputs!$B$57,-Inputs!$B$55),0)</f>
         <v/>
       </c>
     </row>
@@ -4715,43 +4725,43 @@
         <v/>
       </c>
       <c r="C22" s="3">
-        <f>IF(1&lt;=Inputs!$B$56,C19*Inputs!$B$55,0)</f>
+        <f>IF(1&lt;=Inputs!$B$57,C19*Inputs!$B$56,0)</f>
         <v/>
       </c>
       <c r="D22" s="3">
-        <f>IF(2&lt;=Inputs!$B$56,D19*Inputs!$B$55,0)</f>
+        <f>IF(2&lt;=Inputs!$B$57,D19*Inputs!$B$56,0)</f>
         <v/>
       </c>
       <c r="E22" s="3">
-        <f>IF(3&lt;=Inputs!$B$56,E19*Inputs!$B$55,0)</f>
+        <f>IF(3&lt;=Inputs!$B$57,E19*Inputs!$B$56,0)</f>
         <v/>
       </c>
       <c r="F22" s="3">
-        <f>IF(4&lt;=Inputs!$B$56,F19*Inputs!$B$55,0)</f>
+        <f>IF(4&lt;=Inputs!$B$57,F19*Inputs!$B$56,0)</f>
         <v/>
       </c>
       <c r="G22" s="3">
-        <f>IF(5&lt;=Inputs!$B$56,G19*Inputs!$B$55,0)</f>
+        <f>IF(5&lt;=Inputs!$B$57,G19*Inputs!$B$56,0)</f>
         <v/>
       </c>
       <c r="H22" s="3">
-        <f>IF(6&lt;=Inputs!$B$56,H19*Inputs!$B$55,0)</f>
+        <f>IF(6&lt;=Inputs!$B$57,H19*Inputs!$B$56,0)</f>
         <v/>
       </c>
       <c r="I22" s="3">
-        <f>IF(7&lt;=Inputs!$B$56,I19*Inputs!$B$55,0)</f>
+        <f>IF(7&lt;=Inputs!$B$57,I19*Inputs!$B$56,0)</f>
         <v/>
       </c>
       <c r="J22" s="3">
-        <f>IF(8&lt;=Inputs!$B$56,J19*Inputs!$B$55,0)</f>
+        <f>IF(8&lt;=Inputs!$B$57,J19*Inputs!$B$56,0)</f>
         <v/>
       </c>
       <c r="K22" s="3">
-        <f>IF(9&lt;=Inputs!$B$56,K19*Inputs!$B$55,0)</f>
+        <f>IF(9&lt;=Inputs!$B$57,K19*Inputs!$B$56,0)</f>
         <v/>
       </c>
       <c r="L22" s="3">
-        <f>IF(10&lt;=Inputs!$B$56,L19*Inputs!$B$55,0)</f>
+        <f>IF(10&lt;=Inputs!$B$57,L19*Inputs!$B$56,0)</f>
         <v/>
       </c>
     </row>
@@ -5029,43 +5039,43 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>PnL!B17*Inputs!$B$38/365</f>
+        <f>PnL!B17*Inputs!$B$39/365</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>PnL!C17*Inputs!$B$38/365</f>
+        <f>PnL!C17*Inputs!$B$39/365</f>
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>PnL!D17*Inputs!$B$38/365</f>
+        <f>PnL!D17*Inputs!$B$39/365</f>
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>PnL!E17*Inputs!$B$38/365</f>
+        <f>PnL!E17*Inputs!$B$39/365</f>
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>PnL!F17*Inputs!$B$38/365</f>
+        <f>PnL!F17*Inputs!$B$39/365</f>
         <v/>
       </c>
       <c r="G5" s="3">
-        <f>PnL!G17*Inputs!$B$38/365</f>
+        <f>PnL!G17*Inputs!$B$39/365</f>
         <v/>
       </c>
       <c r="H5" s="3">
-        <f>PnL!H17*Inputs!$B$38/365</f>
+        <f>PnL!H17*Inputs!$B$39/365</f>
         <v/>
       </c>
       <c r="I5" s="3">
-        <f>PnL!I17*Inputs!$B$38/365</f>
+        <f>PnL!I17*Inputs!$B$39/365</f>
         <v/>
       </c>
       <c r="J5" s="3">
-        <f>PnL!J17*Inputs!$B$38/365</f>
+        <f>PnL!J17*Inputs!$B$39/365</f>
         <v/>
       </c>
       <c r="K5" s="3">
-        <f>PnL!K17*Inputs!$B$38/365</f>
+        <f>PnL!K17*Inputs!$B$39/365</f>
         <v/>
       </c>
     </row>
@@ -5076,43 +5086,43 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>(PnL!B19+PnL!B20)*Inputs!$B$39/365</f>
+        <f>(PnL!B19+PnL!B20)*Inputs!$B$40/365</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>(PnL!C19+PnL!C20)*Inputs!$B$39/365</f>
+        <f>(PnL!C19+PnL!C20)*Inputs!$B$40/365</f>
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>(PnL!D19+PnL!D20)*Inputs!$B$39/365</f>
+        <f>(PnL!D19+PnL!D20)*Inputs!$B$40/365</f>
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>(PnL!E19+PnL!E20)*Inputs!$B$39/365</f>
+        <f>(PnL!E19+PnL!E20)*Inputs!$B$40/365</f>
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>(PnL!F19+PnL!F20)*Inputs!$B$39/365</f>
+        <f>(PnL!F19+PnL!F20)*Inputs!$B$40/365</f>
         <v/>
       </c>
       <c r="G6" s="3">
-        <f>(PnL!G19+PnL!G20)*Inputs!$B$39/365</f>
+        <f>(PnL!G19+PnL!G20)*Inputs!$B$40/365</f>
         <v/>
       </c>
       <c r="H6" s="3">
-        <f>(PnL!H19+PnL!H20)*Inputs!$B$39/365</f>
+        <f>(PnL!H19+PnL!H20)*Inputs!$B$40/365</f>
         <v/>
       </c>
       <c r="I6" s="3">
-        <f>(PnL!I19+PnL!I20)*Inputs!$B$39/365</f>
+        <f>(PnL!I19+PnL!I20)*Inputs!$B$40/365</f>
         <v/>
       </c>
       <c r="J6" s="3">
-        <f>(PnL!J19+PnL!J20)*Inputs!$B$39/365</f>
+        <f>(PnL!J19+PnL!J20)*Inputs!$B$40/365</f>
         <v/>
       </c>
       <c r="K6" s="3">
-        <f>(PnL!K19+PnL!K20)*Inputs!$B$39/365</f>
+        <f>(PnL!K19+PnL!K20)*Inputs!$B$40/365</f>
         <v/>
       </c>
     </row>
@@ -5123,43 +5133,43 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>(PnL!B32-PnL!B18-PnL!B31-PnL!B21)*Inputs!$B$40/365</f>
+        <f>(PnL!B32-PnL!B18-PnL!B31-PnL!B21)*Inputs!$B$41/365</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>(PnL!C32-PnL!C18-PnL!C31-PnL!C21)*Inputs!$B$40/365</f>
+        <f>(PnL!C32-PnL!C18-PnL!C31-PnL!C21)*Inputs!$B$41/365</f>
         <v/>
       </c>
       <c r="D7" s="3">
-        <f>(PnL!D32-PnL!D18-PnL!D31-PnL!D21)*Inputs!$B$40/365</f>
+        <f>(PnL!D32-PnL!D18-PnL!D31-PnL!D21)*Inputs!$B$41/365</f>
         <v/>
       </c>
       <c r="E7" s="3">
-        <f>(PnL!E32-PnL!E18-PnL!E31-PnL!E21)*Inputs!$B$40/365</f>
+        <f>(PnL!E32-PnL!E18-PnL!E31-PnL!E21)*Inputs!$B$41/365</f>
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>(PnL!F32-PnL!F18-PnL!F31-PnL!F21)*Inputs!$B$40/365</f>
+        <f>(PnL!F32-PnL!F18-PnL!F31-PnL!F21)*Inputs!$B$41/365</f>
         <v/>
       </c>
       <c r="G7" s="3">
-        <f>(PnL!G32-PnL!G18-PnL!G31-PnL!G21)*Inputs!$B$40/365</f>
+        <f>(PnL!G32-PnL!G18-PnL!G31-PnL!G21)*Inputs!$B$41/365</f>
         <v/>
       </c>
       <c r="H7" s="3">
-        <f>(PnL!H32-PnL!H18-PnL!H31-PnL!H21)*Inputs!$B$40/365</f>
+        <f>(PnL!H32-PnL!H18-PnL!H31-PnL!H21)*Inputs!$B$41/365</f>
         <v/>
       </c>
       <c r="I7" s="3">
-        <f>(PnL!I32-PnL!I18-PnL!I31-PnL!I21)*Inputs!$B$40/365</f>
+        <f>(PnL!I32-PnL!I18-PnL!I31-PnL!I21)*Inputs!$B$41/365</f>
         <v/>
       </c>
       <c r="J7" s="3">
-        <f>(PnL!J32-PnL!J18-PnL!J31-PnL!J21)*Inputs!$B$40/365</f>
+        <f>(PnL!J32-PnL!J18-PnL!J31-PnL!J21)*Inputs!$B$41/365</f>
         <v/>
       </c>
       <c r="K7" s="3">
-        <f>(PnL!K32-PnL!K18-PnL!K31-PnL!K21)*Inputs!$B$40/365</f>
+        <f>(PnL!K32-PnL!K18-PnL!K31-PnL!K21)*Inputs!$B$41/365</f>
         <v/>
       </c>
     </row>
@@ -5499,7 +5509,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>Inputs!$B$57+B14</f>
+        <f>Inputs!$B$58+B14</f>
         <v/>
       </c>
       <c r="C15" s="3">
@@ -5546,43 +5556,43 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>MAX(PnL!B33-PnL!B36,0)*Inputs!$B$41*IF(Drivers!B$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!B33-PnL!B36,0)*Inputs!$B$42*IF(Drivers!B$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="C16" s="3">
-        <f>MAX(PnL!C33-PnL!C36,0)*Inputs!$B$41*IF(Drivers!C$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!C33-PnL!C36,0)*Inputs!$B$42*IF(Drivers!C$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="D16" s="3">
-        <f>MAX(PnL!D33-PnL!D36,0)*Inputs!$B$41*IF(Drivers!D$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!D33-PnL!D36,0)*Inputs!$B$42*IF(Drivers!D$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="E16" s="3">
-        <f>MAX(PnL!E33-PnL!E36,0)*Inputs!$B$41*IF(Drivers!E$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!E33-PnL!E36,0)*Inputs!$B$42*IF(Drivers!E$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="F16" s="3">
-        <f>MAX(PnL!F33-PnL!F36,0)*Inputs!$B$41*IF(Drivers!F$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!F33-PnL!F36,0)*Inputs!$B$42*IF(Drivers!F$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="G16" s="3">
-        <f>MAX(PnL!G33-PnL!G36,0)*Inputs!$B$41*IF(Drivers!G$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!G33-PnL!G36,0)*Inputs!$B$42*IF(Drivers!G$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="H16" s="3">
-        <f>MAX(PnL!H33-PnL!H36,0)*Inputs!$B$41*IF(Drivers!H$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!H33-PnL!H36,0)*Inputs!$B$42*IF(Drivers!H$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="I16" s="3">
-        <f>MAX(PnL!I33-PnL!I36,0)*Inputs!$B$41*IF(Drivers!I$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!I33-PnL!I36,0)*Inputs!$B$42*IF(Drivers!I$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="J16" s="3">
-        <f>MAX(PnL!J33-PnL!J36,0)*Inputs!$B$41*IF(Drivers!J$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!J33-PnL!J36,0)*Inputs!$B$42*IF(Drivers!J$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
       <c r="K16" s="3">
-        <f>MAX(PnL!K33-PnL!K36,0)*Inputs!$B$41*IF(Drivers!K$16&lt;Inputs!$B$43,1-Inputs!$B$42,1)</f>
+        <f>MAX(PnL!K33-PnL!K36,0)*Inputs!$B$42*IF(Drivers!K$16&lt;Inputs!$B$44,1-Inputs!$B$43,1)</f>
         <v/>
       </c>
     </row>
@@ -5640,7 +5650,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>-1268200</v>
+        <v>-924720</v>
       </c>
     </row>
     <row r="20">
@@ -5650,7 +5660,7 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>-4033000</v>
+        <v>-3327080</v>
       </c>
     </row>
     <row r="21">
@@ -5660,7 +5670,7 @@
         </is>
       </c>
       <c r="B21" s="3">
-        <f>K17*(1+Inputs!$B$45)/(Inputs!$B$44-Inputs!$B$45)</f>
+        <f>K17*(1+Inputs!$B$46)/(Inputs!$B$45-Inputs!$B$46)</f>
         <v/>
       </c>
     </row>
@@ -5671,7 +5681,7 @@
         </is>
       </c>
       <c r="B22" s="3">
-        <f>B19+B20/(1+Inputs!$B$44)+NPV(Inputs!$B$44,B17:K17)/(1+Inputs!$B$44)</f>
+        <f>B19+B20/(1+Inputs!$B$45)+NPV(Inputs!$B$45,B17:K17)/(1+Inputs!$B$45)</f>
         <v/>
       </c>
     </row>
@@ -5682,7 +5692,7 @@
         </is>
       </c>
       <c r="B23" s="3">
-        <f>B22+B21/(1+Inputs!$B$44)^11</f>
+        <f>B22+B21/(1+Inputs!$B$45)^11</f>
         <v/>
       </c>
     </row>
@@ -5715,7 +5725,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>793109</v>
+        <v>2583075</v>
       </c>
     </row>
   </sheetData>
@@ -5729,7 +5739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5824,40 +5834,40 @@
         <v>4816039.614799246</v>
       </c>
       <c r="C3" t="n">
-        <v>1055514.946085977</v>
+        <v>1144957.798815042</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2192</v>
+        <v>0.2377</v>
       </c>
       <c r="E3" t="n">
-        <v>-2.9875</v>
+        <v>-3.0088</v>
       </c>
       <c r="F3" t="n">
         <v>2029</v>
       </c>
       <c r="G3" t="n">
-        <v>2.0841</v>
+        <v>2.2951</v>
       </c>
       <c r="H3" t="n">
-        <v>-1208100.357020029</v>
+        <v>-806818.3552616632</v>
       </c>
       <c r="I3" t="n">
-        <v>-2943770.350916191</v>
+        <v>-1502654.438202631</v>
       </c>
       <c r="J3" t="n">
-        <v>793108.7364148403</v>
+        <v>2583075.213504797</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1169</v>
+        <v>0.1604</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1283</v>
+        <v>0.1814</v>
       </c>
       <c r="M3" t="n">
-        <v>2672450</v>
+        <v>2011175</v>
       </c>
       <c r="N3" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="4">
@@ -5870,40 +5880,40 @@
         <v>3687996.423313688</v>
       </c>
       <c r="C4" t="n">
-        <v>238518.0559070501</v>
+        <v>338526.5841600737</v>
       </c>
       <c r="D4" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.09180000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>-4.5362</v>
+        <v>-4.8477</v>
       </c>
       <c r="F4" t="n">
         <v>2029</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2544</v>
+        <v>0.5780999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>-5161979.949260596</v>
+        <v>-3700946.650719141</v>
       </c>
       <c r="I4" t="n">
-        <v>-6404199.285283907</v>
+        <v>-4872095.366785241</v>
       </c>
       <c r="J4" t="n">
-        <v>-5796152.501540549</v>
+        <v>-3873944.762915945</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.1169</v>
+        <v>-0.0436</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.1483</v>
+        <v>-0.063</v>
       </c>
       <c r="M4" t="n">
-        <v>2672450</v>
+        <v>2011175</v>
       </c>
       <c r="N4" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="5">
@@ -5916,40 +5926,40 @@
         <v>5516493.202229979</v>
       </c>
       <c r="C5" t="n">
-        <v>1561053.702301371</v>
+        <v>1643938.74190044</v>
       </c>
       <c r="D5" t="n">
-        <v>0.283</v>
+        <v>0.298</v>
       </c>
       <c r="E5" t="n">
-        <v>-2.4878</v>
+        <v>-2.4213</v>
       </c>
       <c r="F5" t="n">
         <v>2029</v>
       </c>
       <c r="G5" t="n">
-        <v>2.6487</v>
+        <v>3.314</v>
       </c>
       <c r="H5" t="n">
-        <v>-407596.1490753151</v>
+        <v>-238985.0049726386</v>
       </c>
       <c r="I5" t="n">
-        <v>-1069699.104642076</v>
+        <v>337982.3078135476</v>
       </c>
       <c r="J5" t="n">
-        <v>4581754.73185224</v>
+        <v>6312687.828744792</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1835</v>
+        <v>0.2278</v>
       </c>
       <c r="L5" t="n">
-        <v>0.2076</v>
+        <v>0.2656</v>
       </c>
       <c r="M5" t="n">
-        <v>2672450</v>
+        <v>2011175</v>
       </c>
       <c r="N5" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="6">
@@ -5962,40 +5972,40 @@
         <v>4734075.662535368</v>
       </c>
       <c r="C6" t="n">
-        <v>994013.4939205484</v>
+        <v>1084275.986172252</v>
       </c>
       <c r="D6" t="n">
-        <v>0.21</v>
+        <v>0.229</v>
       </c>
       <c r="E6" t="n">
-        <v>-3.1969</v>
+        <v>-3.2553</v>
       </c>
       <c r="F6" t="n">
         <v>2029</v>
       </c>
       <c r="G6" t="n">
-        <v>1.9493</v>
+        <v>2.319</v>
       </c>
       <c r="H6" t="n">
-        <v>-1481496.402754171</v>
+        <v>-1025920.212847798</v>
       </c>
       <c r="I6" t="n">
-        <v>-3277640.353375232</v>
+        <v>-1831100.750066701</v>
       </c>
       <c r="J6" t="n">
-        <v>215840.5497608903</v>
+        <v>2014566.386620819</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1047</v>
+        <v>0.1478</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1142</v>
+        <v>0.1663</v>
       </c>
       <c r="M6" t="n">
-        <v>2672450</v>
+        <v>2011175</v>
       </c>
       <c r="N6" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="7">
@@ -6008,86 +6018,86 @@
         <v>4816039.614799246</v>
       </c>
       <c r="C7" t="n">
-        <v>1035801.289384571</v>
+        <v>1129425.82686848</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2151</v>
+        <v>0.2345</v>
       </c>
       <c r="E7" t="n">
-        <v>-3.0062</v>
+        <v>-3.0265</v>
       </c>
       <c r="F7" t="n">
         <v>2029</v>
       </c>
       <c r="G7" t="n">
-        <v>2.0395</v>
+        <v>2.3795</v>
       </c>
       <c r="H7" t="n">
-        <v>-1253846.938489208</v>
+        <v>-828136.8344397454</v>
       </c>
       <c r="I7" t="n">
-        <v>-3370366.237582894</v>
+        <v>-1842591.925497909</v>
       </c>
       <c r="J7" t="n">
-        <v>296357.9864764168</v>
+        <v>2188369.707912541</v>
       </c>
       <c r="K7" t="n">
-        <v>0.1061</v>
+        <v>0.1496</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1153</v>
+        <v>0.1672</v>
       </c>
       <c r="M7" t="n">
-        <v>3076130</v>
+        <v>2334855</v>
       </c>
       <c r="N7" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Construction +20% (build 780/m2)</t>
+          <t>Construction 780/m2 (+30% on lean 600)</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>4816039.614799246</v>
       </c>
       <c r="C8" t="n">
-        <v>1050396.45533086</v>
+        <v>1138815.609908902</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2181</v>
+        <v>0.2365</v>
       </c>
       <c r="E8" t="n">
-        <v>-3.0021</v>
+        <v>-3.0298</v>
       </c>
       <c r="F8" t="n">
         <v>2029</v>
       </c>
       <c r="G8" t="n">
-        <v>2.0725</v>
+        <v>2.3036</v>
       </c>
       <c r="H8" t="n">
-        <v>-1226085.485128762</v>
+        <v>-822577.7247548143</v>
       </c>
       <c r="I8" t="n">
-        <v>-3388167.20880556</v>
+        <v>-2035930.667669875</v>
       </c>
       <c r="J8" t="n">
-        <v>341732.3996247257</v>
+        <v>2041423.609356661</v>
       </c>
       <c r="K8" t="n">
-        <v>0.107</v>
+        <v>0.1447</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1157</v>
+        <v>0.16</v>
       </c>
       <c r="M8" t="n">
-        <v>3124850</v>
+        <v>2554055</v>
       </c>
       <c r="N8" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="9">
@@ -6100,40 +6110,40 @@
         <v>4816039.614799246</v>
       </c>
       <c r="C9" t="n">
-        <v>803178.6333328011</v>
+        <v>919903.7493845164</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1668</v>
+        <v>0.191</v>
       </c>
       <c r="E9" t="n">
-        <v>-3.6602</v>
+        <v>-3.6838</v>
       </c>
       <c r="F9" t="n">
         <v>2029</v>
       </c>
       <c r="G9" t="n">
-        <v>1.5119</v>
+        <v>2.1326</v>
       </c>
       <c r="H9" t="n">
-        <v>-2091986.646320399</v>
+        <v>-1407774.124855621</v>
       </c>
       <c r="I9" t="n">
-        <v>-4106109.710428868</v>
+        <v>-2520875.960361728</v>
       </c>
       <c r="J9" t="n">
-        <v>-1371873.772469816</v>
+        <v>670614.9730338496</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0677</v>
+        <v>0.117</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0716</v>
+        <v>0.1298</v>
       </c>
       <c r="M9" t="n">
-        <v>2672450</v>
+        <v>2011175</v>
       </c>
       <c r="N9" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="10">
@@ -6146,362 +6156,316 @@
         <v>5100583.120829817</v>
       </c>
       <c r="C10" t="n">
-        <v>1255174.193527162</v>
+        <v>1342126.2261579</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2461</v>
+        <v>0.2631</v>
       </c>
       <c r="E10" t="n">
-        <v>-3.7968</v>
+        <v>-3.985</v>
       </c>
       <c r="F10" t="n">
         <v>2029</v>
       </c>
       <c r="G10" t="n">
-        <v>2.1265</v>
+        <v>2.6093</v>
       </c>
       <c r="H10" t="n">
-        <v>-1313070.070748262</v>
+        <v>-979403.2856054966</v>
       </c>
       <c r="I10" t="n">
-        <v>-2681768.450981508</v>
+        <v>-1251698.741220354</v>
       </c>
       <c r="J10" t="n">
-        <v>1744913.833543442</v>
+        <v>3514378.895189697</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1341</v>
+        <v>0.1755</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1469</v>
+        <v>0.1985</v>
       </c>
       <c r="M10" t="n">
-        <v>2672450</v>
+        <v>2011175</v>
       </c>
       <c r="N10" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Land contributed in kind (no purchase)</t>
+          <t>Conditions met: contracted volumes +20%</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4816039.614799246</v>
+        <v>5749977.731373556</v>
       </c>
       <c r="C11" t="n">
-        <v>1055514.946085977</v>
+        <v>1810265.722928906</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2192</v>
+        <v>0.3148</v>
       </c>
       <c r="E11" t="n">
-        <v>-2.9875</v>
+        <v>-2.2255</v>
       </c>
       <c r="F11" t="n">
         <v>2029</v>
       </c>
       <c r="G11" t="n">
-        <v>2.0841</v>
+        <v>3.6536</v>
       </c>
       <c r="H11" t="n">
-        <v>-1208100.357020029</v>
+        <v>-109372.6949971378</v>
       </c>
       <c r="I11" t="n">
-        <v>-2747570.350916191</v>
+        <v>950162.8347123552</v>
       </c>
       <c r="J11" t="n">
-        <v>989308.7364148403</v>
+        <v>7554526.978718204</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1216</v>
+        <v>0.2471</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1345</v>
+        <v>0.2901</v>
       </c>
       <c r="M11" t="n">
-        <v>2476250</v>
+        <v>2011175</v>
       </c>
       <c r="N11" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Conditions met: contracted volumes +20%</t>
+          <t>If MoH requires a general hospital (40 beds, internal medicine + obstetrics)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5749977.731373556</v>
+        <v>5653873.801733973</v>
       </c>
       <c r="C12" t="n">
-        <v>1729566.621039836</v>
+        <v>1037959.904978016</v>
       </c>
       <c r="D12" t="n">
-        <v>0.3008</v>
+        <v>0.1836</v>
       </c>
       <c r="E12" t="n">
-        <v>-2.3213</v>
+        <v>-4.4311</v>
       </c>
       <c r="F12" t="n">
         <v>2029</v>
       </c>
       <c r="G12" t="n">
-        <v>2.9356</v>
+        <v>2.3905</v>
       </c>
       <c r="H12" t="n">
-        <v>-263172.4262964992</v>
+        <v>-1627738.81541511</v>
       </c>
       <c r="I12" t="n">
-        <v>-448720.7892610552</v>
+        <v>-5527063.90782233</v>
       </c>
       <c r="J12" t="n">
-        <v>5840924.63028769</v>
+        <v>-1925167.654288106</v>
       </c>
       <c r="K12" t="n">
-        <v>0.2022</v>
+        <v>0.0664</v>
       </c>
       <c r="L12" t="n">
-        <v>0.2306</v>
+        <v>0.0698</v>
       </c>
       <c r="M12" t="n">
-        <v>2672450</v>
+        <v>5358775</v>
       </c>
       <c r="N12" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>If MoH requires a general hospital (40 beds, internal medicine + obstetrics)</t>
+          <t>F1 CBJ 2.5m + equipment lease 0.5m + equity</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5653873.801733973</v>
+        <v>4816039.614799246</v>
       </c>
       <c r="C13" t="n">
-        <v>939480.7589054862</v>
+        <v>1144957.798815042</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1662</v>
+        <v>0.2377</v>
       </c>
       <c r="E13" t="n">
-        <v>-4.3438</v>
+        <v>-3.0088</v>
       </c>
       <c r="F13" t="n">
         <v>2029</v>
       </c>
       <c r="G13" t="n">
-        <v>1.7683</v>
+        <v>2.2951</v>
       </c>
       <c r="H13" t="n">
-        <v>-2257466.540474215</v>
+        <v>-806818.3552616632</v>
       </c>
       <c r="I13" t="n">
-        <v>-6614213.745913647</v>
+        <v>-1502654.438202631</v>
       </c>
       <c r="J13" t="n">
-        <v>-3406012.032578514</v>
+        <v>2583075.213504797</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0411</v>
+        <v>0.1604</v>
       </c>
       <c r="L13" t="n">
-        <v>0.0421</v>
+        <v>0.1814</v>
       </c>
       <c r="M13" t="n">
-        <v>5480050</v>
+        <v>2011175</v>
       </c>
       <c r="N13" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>F1 CBJ 3.0m + equipment lease 0.6m + equity</t>
+          <t>F2 CBJ 2.5m + Islamic ijara 1.2m + lease 0.5m + equity</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>4816039.614799246</v>
       </c>
       <c r="C14" t="n">
-        <v>1055514.946085977</v>
+        <v>1144957.798815042</v>
       </c>
       <c r="D14" t="n">
-        <v>0.2192</v>
+        <v>0.2377</v>
       </c>
       <c r="E14" t="n">
-        <v>-2.9875</v>
+        <v>-2.123</v>
       </c>
       <c r="F14" t="n">
         <v>2029</v>
       </c>
       <c r="G14" t="n">
-        <v>2.0841</v>
+        <v>1.6049</v>
       </c>
       <c r="H14" t="n">
-        <v>-1208100.357020029</v>
+        <v>-1389033.695892893</v>
       </c>
       <c r="I14" t="n">
-        <v>-2943770.350916191</v>
+        <v>-1502654.438202631</v>
       </c>
       <c r="J14" t="n">
-        <v>793108.7364148403</v>
+        <v>2583075.213504797</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1169</v>
+        <v>0.1604</v>
       </c>
       <c r="L14" t="n">
-        <v>0.1283</v>
+        <v>0.2014</v>
       </c>
       <c r="M14" t="n">
-        <v>2672450</v>
+        <v>862175</v>
       </c>
       <c r="N14" t="n">
-        <v>3600000</v>
+        <v>4200000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>F2 CBJ 3.0m + Islamic ijara 1.2m + lease 0.6m + equity</t>
+          <t>F3 Commercial loan only 3.6m at 8.5% (no CBJ)</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>4816039.614799246</v>
       </c>
       <c r="C15" t="n">
-        <v>1055514.946085977</v>
+        <v>1144957.798815042</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2192</v>
+        <v>0.2377</v>
       </c>
       <c r="E15" t="n">
-        <v>-2.2167</v>
+        <v>0.0412</v>
       </c>
       <c r="F15" t="n">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="G15" t="n">
-        <v>1.423</v>
+        <v>1.5802</v>
       </c>
       <c r="H15" t="n">
-        <v>-1927833.315741536</v>
+        <v>-1221568.143481991</v>
       </c>
       <c r="I15" t="n">
-        <v>-2943770.350916191</v>
+        <v>-1502654.438202631</v>
       </c>
       <c r="J15" t="n">
-        <v>793108.7364148403</v>
+        <v>2583075.213504797</v>
       </c>
       <c r="K15" t="n">
-        <v>0.1169</v>
+        <v>0.1604</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1357</v>
+        <v>0.1746</v>
       </c>
       <c r="M15" t="n">
-        <v>1523450</v>
+        <v>1522800</v>
       </c>
       <c r="N15" t="n">
-        <v>4800000</v>
+        <v>3600000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>F3 Commercial loan only 3.6m at 8.5% (no CBJ)</t>
+          <t>F4 Doctor-investor company: CBJ 2.0m + lease 0.5m, more equity from 10-15 doctors</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>4816039.614799246</v>
       </c>
       <c r="C16" t="n">
-        <v>1055514.946085977</v>
+        <v>1144957.798815042</v>
       </c>
       <c r="D16" t="n">
-        <v>0.2192</v>
+        <v>0.2377</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1109</v>
+        <v>-3.2953</v>
       </c>
       <c r="F16" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="G16" t="n">
-        <v>1.4397</v>
+        <v>2.8617</v>
       </c>
       <c r="H16" t="n">
-        <v>-1408448.223233431</v>
+        <v>-641069.9638005851</v>
       </c>
       <c r="I16" t="n">
-        <v>-2943770.350916191</v>
+        <v>-1502654.438202631</v>
       </c>
       <c r="J16" t="n">
-        <v>793108.7364148403</v>
+        <v>2583075.213504797</v>
       </c>
       <c r="K16" t="n">
-        <v>0.1169</v>
+        <v>0.1604</v>
       </c>
       <c r="L16" t="n">
-        <v>0.1146</v>
+        <v>0.1732</v>
       </c>
       <c r="M16" t="n">
-        <v>2772200</v>
+        <v>2499300</v>
       </c>
       <c r="N16" t="n">
-        <v>3600000</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>F4 Doctor-investor company: CBJ 2.0m + lease 0.6m, equity from 10-15 doctors</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>4816039.614799246</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1055514.946085977</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.2192</v>
-      </c>
-      <c r="E17" t="n">
-        <v>-3.4936</v>
-      </c>
-      <c r="F17" t="n">
-        <v>2029</v>
-      </c>
-      <c r="G17" t="n">
-        <v>3.1261</v>
-      </c>
-      <c r="H17" t="n">
-        <v>-813562.7648176152</v>
-      </c>
-      <c r="I17" t="n">
-        <v>-2943770.350916191</v>
-      </c>
-      <c r="J17" t="n">
-        <v>793108.7364148403</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0.1169</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0.1202</v>
-      </c>
-      <c r="M17" t="n">
-        <v>3648700</v>
-      </c>
-      <c r="N17" t="n">
-        <v>2600000</v>
+        <v>2500000</v>
       </c>
     </row>
   </sheetData>
@@ -6543,7 +6507,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>This study (20 beds)</t>
+          <t>This study (20 beds, lean Phase 1)</t>
         </is>
       </c>
     </row>
@@ -6557,7 +6521,7 @@
         <v>7574640</v>
       </c>
       <c r="C4" t="n">
-        <v>6272450</v>
+        <v>5011175</v>
       </c>
     </row>
     <row r="5">
@@ -6570,7 +6534,7 @@
         <v>94683</v>
       </c>
       <c r="C5" t="n">
-        <v>313622</v>
+        <v>250559</v>
       </c>
     </row>
     <row r="6">
@@ -6583,7 +6547,7 @@
         <v>298</v>
       </c>
       <c r="C6" t="n">
-        <v>650</v>
+        <v>600</v>
       </c>
     </row>
     <row r="7">
@@ -6596,7 +6560,7 @@
         <v>3150400</v>
       </c>
       <c r="C7" t="n">
-        <v>1650000</v>
+        <v>1300000</v>
       </c>
     </row>
     <row r="8">
@@ -6609,7 +6573,7 @@
         <v>100</v>
       </c>
       <c r="C8" t="n">
-        <v>117</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9">
@@ -6622,7 +6586,7 @@
         <v>609960</v>
       </c>
       <c r="C9" t="n">
-        <v>1160893</v>
+        <v>970668</v>
       </c>
     </row>
     <row r="10">
@@ -6635,7 +6599,7 @@
         <v>508</v>
       </c>
       <c r="C10" t="n">
-        <v>1034</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="11">
@@ -6680,7 +6644,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="14">
@@ -6710,7 +6674,7 @@
         <v>150054</v>
       </c>
       <c r="C15" t="n">
-        <v>-925391</v>
+        <v>-703566</v>
       </c>
     </row>
   </sheetData>

</xml_diff>